<commit_message>
add ablation; initial plots
</commit_message>
<xml_diff>
--- a/ArrayExpress/1-s2.0-S0969996120305003-mmc2.xlsx
+++ b/ArrayExpress/1-s2.0-S0969996120305003-mmc2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/owensun/Downloads/code/finding-datasets-with-LLMs/ArrayExpress/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B59CCEC7-35E5-5249-A413-EA68D831DB08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AE6765A-994E-2F47-8AF7-963704ED4851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6380" yWindow="600" windowWidth="24480" windowHeight="15320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="15320" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Systematic Search Criteria" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'AD Datasets'!$D$2:$D$78</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ALS-FTD Datasets'!$D$2:$D$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ALS-FTD Datasets'!$A$2:$N$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'LBD Datasets'!$D$2:$D$90</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -2570,6 +2570,21 @@
     <xf numFmtId="0" fontId="10" fillId="15" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2582,24 +2597,33 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2611,30 +2635,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -8468,7 +8468,7 @@
         <v>20</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>1</v>
+        <v>465</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>3</v>
@@ -8550,7 +8550,7 @@
         <v>E-MTAB-8635: Gene expression profiles in spinal cord of control and sporadic Amyotrophic Lateral Sclerosis patients</v>
       </c>
     </row>
-    <row r="4" spans="1:17" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="70">
         <v>2</v>
       </c>
@@ -8580,20 +8580,20 @@
       </c>
     </row>
     <row r="5" spans="1:17" s="43" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="107">
+      <c r="A5" s="112">
         <v>3</v>
       </c>
-      <c r="B5" s="107" t="s">
+      <c r="B5" s="112" t="s">
         <v>184</v>
       </c>
-      <c r="C5" s="106" t="s">
+      <c r="C5" s="111" t="s">
         <v>465</v>
       </c>
-      <c r="D5" s="108"/>
-      <c r="E5" s="109" t="s">
+      <c r="D5" s="113"/>
+      <c r="E5" s="114" t="s">
         <v>251</v>
       </c>
-      <c r="F5" s="106" t="s">
+      <c r="F5" s="111" t="s">
         <v>487</v>
       </c>
       <c r="G5" s="41" t="s">
@@ -8608,27 +8608,27 @@
       <c r="J5" s="39">
         <v>10</v>
       </c>
-      <c r="K5" s="110">
+      <c r="K5" s="106">
         <v>42831</v>
       </c>
-      <c r="L5" s="111" t="s">
+      <c r="L5" s="107" t="s">
         <v>492</v>
       </c>
-      <c r="M5" s="111" t="s">
+      <c r="M5" s="107" t="s">
         <v>470</v>
       </c>
-      <c r="N5" s="112" t="str">
+      <c r="N5" s="108" t="str">
         <f t="shared" si="0"/>
         <v>E-MTAB-6189: Differential gene expression study in brain samples from patients suffering distinct frontotemporal lobar degeneration (FTLD) conditions</v>
       </c>
     </row>
-    <row r="6" spans="1:17" s="37" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="107"/>
-      <c r="B6" s="107"/>
-      <c r="C6" s="106"/>
-      <c r="D6" s="108"/>
-      <c r="E6" s="109"/>
-      <c r="F6" s="106"/>
+    <row r="6" spans="1:17" s="37" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="112"/>
+      <c r="B6" s="112"/>
+      <c r="C6" s="111"/>
+      <c r="D6" s="113"/>
+      <c r="E6" s="114"/>
+      <c r="F6" s="111"/>
       <c r="G6" s="41" t="s">
         <v>491</v>
       </c>
@@ -8641,10 +8641,10 @@
       <c r="J6" s="39">
         <v>10</v>
       </c>
-      <c r="K6" s="110"/>
-      <c r="L6" s="111"/>
-      <c r="M6" s="111"/>
-      <c r="N6" s="113"/>
+      <c r="K6" s="106"/>
+      <c r="L6" s="107"/>
+      <c r="M6" s="107"/>
+      <c r="N6" s="109"/>
     </row>
     <row r="7" spans="1:17" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="70">
@@ -8762,7 +8762,7 @@
         <v>E-GEOD-68605: C9ORF72 GGGGCC expanded repeats produce splicing dysregulation which correlates with disease severity in amyotrophic lateral sclerosis [HG-U133_Plus_2]</v>
       </c>
     </row>
-    <row r="11" spans="1:17" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="70">
         <v>8</v>
       </c>
@@ -8791,7 +8791,7 @@
         <v>E-GEOD-59128: The human airway epithelial basal cell transcriptome in the early response to injury</v>
       </c>
     </row>
-    <row r="12" spans="1:17" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="70">
         <v>9</v>
       </c>
@@ -8820,7 +8820,7 @@
         <v>E-GEOD-68240: hiPSC-derived motor neurons: sporadic ALS patients vs. controls</v>
       </c>
     </row>
-    <row r="13" spans="1:17" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="70">
         <v>10</v>
       </c>
@@ -8849,7 +8849,7 @@
         <v>E-GEOD-60082: Effective sorafenib treatment response in a panel of genomically-characterized malignant peripheral nerve sheath tumor orthoxenograft models</v>
       </c>
     </row>
-    <row r="14" spans="1:17" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="70">
         <v>11</v>
       </c>
@@ -9008,7 +9008,7 @@
         <v>E-GEOD-58316: Suppression of NCALD protects against spinal muscular atrophy by restoring impaired endocytosis</v>
       </c>
     </row>
-    <row r="19" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="70">
         <v>16</v>
       </c>
@@ -9037,7 +9037,7 @@
         <v>E-GEOD-40807: MiRNA expression profiling in human medullary thyroid carcinoma</v>
       </c>
     </row>
-    <row r="20" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="70">
         <v>17</v>
       </c>
@@ -9066,7 +9066,7 @@
         <v>E-GEOD-44721: IL4 DCs and monocytes stimulated by 13 human vaccines and LPS for 6hr</v>
       </c>
     </row>
-    <row r="21" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="70">
         <v>18</v>
       </c>
@@ -9356,7 +9356,7 @@
         <v>E-GEOD-52392: Integrative DNA methylation and gene expression analysis in high-grade soft tissue sarcomas</v>
       </c>
     </row>
-    <row r="31" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="70">
         <v>28</v>
       </c>
@@ -9385,7 +9385,7 @@
         <v>E-GEOD-52390: Integrative DNA methylation and gene expression analysis in high-grade soft tissue sarcomas [gene expression]</v>
       </c>
     </row>
-    <row r="32" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="70">
         <v>29</v>
       </c>
@@ -9414,7 +9414,7 @@
         <v>E-MTAB-1927: Transcription profiling by array of neurons differentiated from induced pluripotent stem cells carrying a mutation in the SOD1 gene, an expanded GGGGCC repeat mutation in the chromosome 9 open reading frame 72 gene and those without any (control)</v>
       </c>
     </row>
-    <row r="33" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="70">
         <v>30</v>
       </c>
@@ -9542,7 +9542,7 @@
         <v>E-GEOD-49657: The inducuction of UPR target genes in response to zinc depletion and serum starvation in HeLa cells</v>
       </c>
     </row>
-    <row r="37" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="70">
         <v>34</v>
       </c>
@@ -9629,7 +9629,7 @@
         <v>E-GEOD-40438: Gene expression profiling of resistant and vulnerable motor neuron subtypes in amyotrophic lateral sclerosis</v>
       </c>
     </row>
-    <row r="40" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="70">
         <v>37</v>
       </c>
@@ -9774,7 +9774,7 @@
         <v>E-GEOD-31243: Transcriptional Alterations of Hamstring Muscle Contractures in Children with Cerebral Palsy</v>
       </c>
     </row>
-    <row r="45" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="70">
         <v>42</v>
       </c>
@@ -9861,7 +9861,7 @@
         <v>E-GEOD-39644: Amyotrophic lateral sclerosis</v>
       </c>
     </row>
-    <row r="48" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="70">
         <v>45</v>
       </c>
@@ -9948,7 +9948,7 @@
         <v>E-GEOD-30806: Expression profiling in VCP-associated myopathy</v>
       </c>
     </row>
-    <row r="51" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="70">
         <v>48</v>
       </c>
@@ -9977,7 +9977,7 @@
         <v>E-GEOD-27564: Gene expression profiles of subepithelial myofibroblasts from mouse ileum or colon, implanted together with human cancer cells in mouse xenografts</v>
       </c>
     </row>
-    <row r="52" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="70">
         <v>49</v>
       </c>
@@ -10065,20 +10065,20 @@
       </c>
     </row>
     <row r="55" spans="1:14" s="43" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="107">
+      <c r="A55" s="112">
         <v>52</v>
       </c>
-      <c r="B55" s="107" t="s">
+      <c r="B55" s="112" t="s">
         <v>77</v>
       </c>
-      <c r="C55" s="106" t="s">
+      <c r="C55" s="111" t="s">
         <v>465</v>
       </c>
-      <c r="D55" s="108"/>
-      <c r="E55" s="109" t="s">
+      <c r="D55" s="113"/>
+      <c r="E55" s="114" t="s">
         <v>153</v>
       </c>
-      <c r="F55" s="106" t="s">
+      <c r="F55" s="111" t="s">
         <v>466</v>
       </c>
       <c r="G55" s="76" t="s">
@@ -10093,27 +10093,27 @@
       <c r="J55" s="39">
         <v>4</v>
       </c>
-      <c r="K55" s="110">
+      <c r="K55" s="106">
         <v>40774</v>
       </c>
-      <c r="L55" s="111" t="s">
+      <c r="L55" s="107" t="s">
         <v>469</v>
       </c>
-      <c r="M55" s="111" t="s">
+      <c r="M55" s="107" t="s">
         <v>470</v>
       </c>
-      <c r="N55" s="112" t="str">
+      <c r="N55" s="108" t="str">
         <f t="shared" si="0"/>
         <v>E-MTAB-656: Alternative splicing in human temporal cortex</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="107"/>
-      <c r="B56" s="107"/>
-      <c r="C56" s="106"/>
-      <c r="D56" s="108"/>
-      <c r="E56" s="109"/>
-      <c r="F56" s="106"/>
+    <row r="56" spans="1:14" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="112"/>
+      <c r="B56" s="112"/>
+      <c r="C56" s="111"/>
+      <c r="D56" s="113"/>
+      <c r="E56" s="114"/>
+      <c r="F56" s="111"/>
       <c r="G56" s="76" t="s">
         <v>500</v>
       </c>
@@ -10126,18 +10126,18 @@
       <c r="J56" s="39">
         <v>3</v>
       </c>
-      <c r="K56" s="110"/>
-      <c r="L56" s="111"/>
-      <c r="M56" s="111"/>
-      <c r="N56" s="114"/>
-    </row>
-    <row r="57" spans="1:14" s="37" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="107"/>
-      <c r="B57" s="107"/>
-      <c r="C57" s="106"/>
-      <c r="D57" s="108"/>
-      <c r="E57" s="109"/>
-      <c r="F57" s="106"/>
+      <c r="K56" s="106"/>
+      <c r="L56" s="107"/>
+      <c r="M56" s="107"/>
+      <c r="N56" s="110"/>
+    </row>
+    <row r="57" spans="1:14" s="37" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="112"/>
+      <c r="B57" s="112"/>
+      <c r="C57" s="111"/>
+      <c r="D57" s="113"/>
+      <c r="E57" s="114"/>
+      <c r="F57" s="111"/>
       <c r="G57" s="76" t="s">
         <v>501</v>
       </c>
@@ -10150,10 +10150,10 @@
       <c r="J57" s="39">
         <v>3</v>
       </c>
-      <c r="K57" s="110"/>
-      <c r="L57" s="111"/>
-      <c r="M57" s="111"/>
-      <c r="N57" s="113"/>
+      <c r="K57" s="106"/>
+      <c r="L57" s="107"/>
+      <c r="M57" s="107"/>
+      <c r="N57" s="109"/>
     </row>
     <row r="58" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="70">
@@ -10242,7 +10242,7 @@
         <v>E-GEOD-20589: Microarray analysis identifies the gene signature of surviving motor neurons in human SOD1-related motor neuron disease</v>
       </c>
     </row>
-    <row r="61" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="70">
         <v>56</v>
       </c>
@@ -10300,7 +10300,7 @@
         <v>E-GEOD-21450: Dysregulated expression and alternative splicing of genes controlling neuritogenesis and axon guidance revealed by exon-sensitive microarrays in models of neurodegeneration</v>
       </c>
     </row>
-    <row r="63" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="70">
         <v>58</v>
       </c>
@@ -10329,7 +10329,7 @@
         <v>E-GEOD-21298: Profiling wt SOD versus ALS SOD1(G93A) mutant</v>
       </c>
     </row>
-    <row r="64" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="70">
         <v>59</v>
       </c>
@@ -10459,7 +10459,7 @@
         <v>E-MEXP-2280: Transcription profiling of patients with four neurodegenerative disorders distinguishes tauopathies and identifies shared molecular pathways</v>
       </c>
     </row>
-    <row r="68" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="70">
         <v>63</v>
       </c>
@@ -10517,7 +10517,7 @@
         <v>E-GEOD-13828: Transcription profiling of human spinal muscular atrophy patient induced pluripotent stem cells</v>
       </c>
     </row>
-    <row r="70" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="70">
         <v>65</v>
       </c>
@@ -10575,7 +10575,7 @@
         <v>E-GEOD-13162: Transcription profiling of human postmortem brain samples with and without FTLD-U</v>
       </c>
     </row>
-    <row r="72" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="70">
         <v>67</v>
       </c>
@@ -10633,7 +10633,7 @@
         <v>E-GEOD-9397: Transcription profiling of human Facioscapulohumeral muscular dystrophy (FSHD) muscle profiles</v>
       </c>
     </row>
-    <row r="74" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="70">
         <v>69</v>
       </c>
@@ -10691,7 +10691,7 @@
         <v>E-GEOD-4595: Transcription profiling of human motor cortex in sporadic amyotrophic lateral sclerosis</v>
       </c>
     </row>
-    <row r="76" spans="1:14" s="38" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:14" s="38" customFormat="1" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="70">
         <v>71</v>
       </c>
@@ -10935,25 +10935,14 @@
     <row r="202" ht="13.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="203" ht="13.5" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <autoFilter ref="D2:D79" xr:uid="{8A4DBBA3-BCD7-4B76-8A5E-7D4B96E190C3}">
-    <filterColumn colId="0">
-      <filters blank="1">
-        <filter val="Cell-Line or Other Disease Model"/>
-        <filter val="Not Brain Tissue"/>
-        <filter val="Not Disease in Question"/>
-        <filter val="Not Human"/>
+  <autoFilter ref="A2:N79" xr:uid="{FD0C3308-226C-4DF5-9177-C79A3165AADB}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Yes"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <mergeCells count="20">
-    <mergeCell ref="K55:K57"/>
-    <mergeCell ref="L55:L57"/>
-    <mergeCell ref="M55:M57"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="N55:N57"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="M5:M6"/>
     <mergeCell ref="F55:F57"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="B5:B6"/>
@@ -10966,6 +10955,14 @@
     <mergeCell ref="C55:C57"/>
     <mergeCell ref="D55:D57"/>
     <mergeCell ref="E55:E57"/>
+    <mergeCell ref="K55:K57"/>
+    <mergeCell ref="L55:L57"/>
+    <mergeCell ref="M55:M57"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="N55:N57"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="M5:M6"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D5 D7:D55 D58:D1048576" xr:uid="{71126AA8-AB99-4150-93E4-CC5B4992ABDD}">
@@ -11076,20 +11073,20 @@
     </row>
     <row r="4" spans="1:16" s="60" customFormat="1" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="81"/>
-      <c r="B4" s="123" t="s">
+      <c r="B4" s="118" t="s">
         <v>506</v>
       </c>
-      <c r="C4" s="124"/>
-      <c r="D4" s="124"/>
-      <c r="E4" s="124"/>
-      <c r="F4" s="124"/>
-      <c r="G4" s="124"/>
-      <c r="H4" s="124"/>
-      <c r="I4" s="124"/>
-      <c r="J4" s="124"/>
-      <c r="K4" s="124"/>
-      <c r="L4" s="124"/>
-      <c r="M4" s="125"/>
+      <c r="C4" s="119"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="119"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="119"/>
+      <c r="H4" s="119"/>
+      <c r="I4" s="119"/>
+      <c r="J4" s="119"/>
+      <c r="K4" s="119"/>
+      <c r="L4" s="119"/>
+      <c r="M4" s="120"/>
     </row>
     <row r="5" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="78">
@@ -11186,20 +11183,20 @@
     </row>
     <row r="8" spans="1:16" s="60" customFormat="1" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="82"/>
-      <c r="B8" s="120" t="s">
+      <c r="B8" s="115" t="s">
         <v>512</v>
       </c>
-      <c r="C8" s="121"/>
-      <c r="D8" s="121"/>
-      <c r="E8" s="121"/>
-      <c r="F8" s="121"/>
-      <c r="G8" s="121"/>
-      <c r="H8" s="121"/>
-      <c r="I8" s="121"/>
-      <c r="J8" s="121"/>
-      <c r="K8" s="121"/>
-      <c r="L8" s="121"/>
-      <c r="M8" s="122"/>
+      <c r="C8" s="116"/>
+      <c r="D8" s="116"/>
+      <c r="E8" s="116"/>
+      <c r="F8" s="116"/>
+      <c r="G8" s="116"/>
+      <c r="H8" s="116"/>
+      <c r="I8" s="116"/>
+      <c r="J8" s="116"/>
+      <c r="K8" s="116"/>
+      <c r="L8" s="116"/>
+      <c r="M8" s="117"/>
     </row>
     <row r="9" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="78">
@@ -11296,20 +11293,20 @@
     </row>
     <row r="12" spans="1:16" s="60" customFormat="1" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="82"/>
-      <c r="B12" s="117" t="s">
+      <c r="B12" s="125" t="s">
         <v>507</v>
       </c>
-      <c r="C12" s="118"/>
-      <c r="D12" s="118"/>
-      <c r="E12" s="118"/>
-      <c r="F12" s="118"/>
-      <c r="G12" s="118"/>
-      <c r="H12" s="118"/>
-      <c r="I12" s="118"/>
-      <c r="J12" s="118"/>
-      <c r="K12" s="118"/>
-      <c r="L12" s="118"/>
-      <c r="M12" s="119"/>
+      <c r="C12" s="126"/>
+      <c r="D12" s="126"/>
+      <c r="E12" s="126"/>
+      <c r="F12" s="126"/>
+      <c r="G12" s="126"/>
+      <c r="H12" s="126"/>
+      <c r="I12" s="126"/>
+      <c r="J12" s="126"/>
+      <c r="K12" s="126"/>
+      <c r="L12" s="126"/>
+      <c r="M12" s="127"/>
     </row>
     <row r="13" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="78">
@@ -11352,16 +11349,16 @@
     </row>
     <row r="14" spans="1:16" s="59" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="82"/>
-      <c r="B14" s="126">
+      <c r="B14" s="121">
         <v>3</v>
       </c>
-      <c r="C14" s="107" t="s">
+      <c r="C14" s="112" t="s">
         <v>184</v>
       </c>
-      <c r="D14" s="109" t="s">
+      <c r="D14" s="114" t="s">
         <v>251</v>
       </c>
-      <c r="E14" s="106" t="s">
+      <c r="E14" s="111" t="s">
         <v>487</v>
       </c>
       <c r="F14" s="41" t="s">
@@ -11376,26 +11373,26 @@
       <c r="I14" s="39">
         <v>10</v>
       </c>
-      <c r="J14" s="110">
+      <c r="J14" s="106">
         <v>42831</v>
       </c>
-      <c r="K14" s="111" t="s">
+      <c r="K14" s="107" t="s">
         <v>492</v>
       </c>
-      <c r="L14" s="111" t="s">
+      <c r="L14" s="107" t="s">
         <v>470</v>
       </c>
-      <c r="M14" s="115" t="str">
+      <c r="M14" s="122" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://www.ebi.ac.uk/arrayexpress/experiments/",C14), _xlfn.CONCAT(C14, ": ", D14))</f>
         <v>E-MTAB-6189: Differential gene expression study in brain samples from patients suffering distinct frontotemporal lobar degeneration (FTLD) conditions</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="83"/>
-      <c r="B15" s="126"/>
-      <c r="C15" s="107"/>
-      <c r="D15" s="109"/>
-      <c r="E15" s="106"/>
+      <c r="B15" s="121"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="114"/>
+      <c r="E15" s="111"/>
       <c r="F15" s="41" t="s">
         <v>491</v>
       </c>
@@ -11408,10 +11405,10 @@
       <c r="I15" s="39">
         <v>10</v>
       </c>
-      <c r="J15" s="110"/>
-      <c r="K15" s="111"/>
-      <c r="L15" s="111"/>
-      <c r="M15" s="116"/>
+      <c r="J15" s="106"/>
+      <c r="K15" s="107"/>
+      <c r="L15" s="107"/>
+      <c r="M15" s="124"/>
     </row>
     <row r="16" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="83"/>
@@ -11493,16 +11490,16 @@
     </row>
     <row r="18" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="83"/>
-      <c r="B18" s="126">
+      <c r="B18" s="121">
         <v>52</v>
       </c>
-      <c r="C18" s="107" t="s">
+      <c r="C18" s="112" t="s">
         <v>77</v>
       </c>
-      <c r="D18" s="109" t="s">
+      <c r="D18" s="114" t="s">
         <v>153</v>
       </c>
-      <c r="E18" s="106" t="s">
+      <c r="E18" s="111" t="s">
         <v>466</v>
       </c>
       <c r="F18" s="76" t="s">
@@ -11517,26 +11514,26 @@
       <c r="I18" s="39">
         <v>4</v>
       </c>
-      <c r="J18" s="110">
+      <c r="J18" s="106">
         <v>40774</v>
       </c>
-      <c r="K18" s="111" t="s">
+      <c r="K18" s="107" t="s">
         <v>469</v>
       </c>
-      <c r="L18" s="111" t="s">
+      <c r="L18" s="107" t="s">
         <v>470</v>
       </c>
-      <c r="M18" s="115" t="str">
+      <c r="M18" s="122" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://www.ebi.ac.uk/arrayexpress/experiments/",C18), _xlfn.CONCAT(C18, ": ", D18))</f>
         <v>E-MTAB-656: Alternative splicing in human temporal cortex</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="83"/>
-      <c r="B19" s="126"/>
-      <c r="C19" s="107"/>
-      <c r="D19" s="109"/>
-      <c r="E19" s="106"/>
+      <c r="B19" s="121"/>
+      <c r="C19" s="112"/>
+      <c r="D19" s="114"/>
+      <c r="E19" s="111"/>
       <c r="F19" s="76" t="s">
         <v>500</v>
       </c>
@@ -11549,17 +11546,17 @@
       <c r="I19" s="39">
         <v>3</v>
       </c>
-      <c r="J19" s="110"/>
-      <c r="K19" s="111"/>
-      <c r="L19" s="111"/>
-      <c r="M19" s="127"/>
+      <c r="J19" s="106"/>
+      <c r="K19" s="107"/>
+      <c r="L19" s="107"/>
+      <c r="M19" s="123"/>
     </row>
     <row r="20" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="83"/>
-      <c r="B20" s="126"/>
-      <c r="C20" s="107"/>
-      <c r="D20" s="109"/>
-      <c r="E20" s="106"/>
+      <c r="B20" s="121"/>
+      <c r="C20" s="112"/>
+      <c r="D20" s="114"/>
+      <c r="E20" s="111"/>
       <c r="F20" s="76" t="s">
         <v>501</v>
       </c>
@@ -11572,10 +11569,10 @@
       <c r="I20" s="39">
         <v>3</v>
       </c>
-      <c r="J20" s="110"/>
-      <c r="K20" s="111"/>
-      <c r="L20" s="111"/>
-      <c r="M20" s="116"/>
+      <c r="J20" s="106"/>
+      <c r="K20" s="107"/>
+      <c r="L20" s="107"/>
+      <c r="M20" s="124"/>
     </row>
     <row r="21" spans="1:13" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="83"/>
@@ -11703,6 +11700,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="J18:J20"/>
+    <mergeCell ref="B12:M12"/>
     <mergeCell ref="B8:M8"/>
     <mergeCell ref="B4:M4"/>
     <mergeCell ref="B18:B20"/>
@@ -11719,9 +11719,6 @@
     <mergeCell ref="J14:J15"/>
     <mergeCell ref="K14:K15"/>
     <mergeCell ref="L14:L15"/>
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="J18:J20"/>
-    <mergeCell ref="B12:M12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>

</xml_diff>